<commit_message>
Archivos importados del repo del servidor para los cambios
</commit_message>
<xml_diff>
--- a/registros.xlsx
+++ b/registros.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="70">
   <si>
     <t>Fecha</t>
   </si>
@@ -200,6 +200,27 @@
   </si>
   <si>
     <t>galicia</t>
+  </si>
+  <si>
+    <t>5/8/2026, 10:40:46 p.m.</t>
+  </si>
+  <si>
+    <t>043e053c-aff6-4eee-9a79-01fdbebe9908</t>
+  </si>
+  <si>
+    <t>Abigail Sánchez</t>
+  </si>
+  <si>
+    <t>555555555555555555</t>
+  </si>
+  <si>
+    <t>abigail.sanchez@cua.uam.mx</t>
+  </si>
+  <si>
+    <t>edo mex</t>
+  </si>
+  <si>
+    <t>21</t>
   </si>
 </sst>
 </file>
@@ -585,7 +606,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="20" customWidth="1"/>
@@ -946,6 +967,38 @@
         <v>13</v>
       </c>
     </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" t="s">
+        <v>64</v>
+      </c>
+      <c r="D12" t="s">
+        <v>65</v>
+      </c>
+      <c r="E12" t="s">
+        <v>66</v>
+      </c>
+      <c r="F12" t="s">
+        <v>67</v>
+      </c>
+      <c r="G12" t="s">
+        <v>68</v>
+      </c>
+      <c r="H12" t="s">
+        <v>69</v>
+      </c>
+      <c r="I12" t="s">
+        <v>44</v>
+      </c>
+      <c r="J12" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>

<commit_message>
Cambio de colores del panel y soporte de imágenes y PDF
</commit_message>
<xml_diff>
--- a/registros.xlsx
+++ b/registros.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="79">
   <si>
     <t>Fecha</t>
   </si>
@@ -221,6 +221,33 @@
   </si>
   <si>
     <t>21</t>
+  </si>
+  <si>
+    <t>2/10/2026, 11:43:35 p.m.</t>
+  </si>
+  <si>
+    <t>5c11188f-7e46-4a70-8fd0-6445b3f5d706</t>
+  </si>
+  <si>
+    <t>5518956452</t>
+  </si>
+  <si>
+    <t>daniela.ejemplo@gmail.com</t>
+  </si>
+  <si>
+    <t>servicioSolicita: Atención psicológica | ingresoMensual: menos de 5000 | dependientesEconomicos: 0</t>
+  </si>
+  <si>
+    <t>2/10/2026, 11:51:15 p.m.</t>
+  </si>
+  <si>
+    <t>daniela nava</t>
+  </si>
+  <si>
+    <t>5578954612</t>
+  </si>
+  <si>
+    <t>daniela.nava@cua.uam.mx</t>
   </si>
 </sst>
 </file>
@@ -606,7 +633,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="20" customWidth="1"/>
@@ -999,6 +1026,70 @@
         <v>13</v>
       </c>
     </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" t="s">
+        <v>71</v>
+      </c>
+      <c r="D13" t="s">
+        <v>25</v>
+      </c>
+      <c r="E13" t="s">
+        <v>72</v>
+      </c>
+      <c r="F13" t="s">
+        <v>73</v>
+      </c>
+      <c r="G13" t="s">
+        <v>49</v>
+      </c>
+      <c r="H13" t="s">
+        <v>43</v>
+      </c>
+      <c r="I13" t="s">
+        <v>13</v>
+      </c>
+      <c r="J13" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>75</v>
+      </c>
+      <c r="B14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C14" t="s">
+        <v>71</v>
+      </c>
+      <c r="D14" t="s">
+        <v>76</v>
+      </c>
+      <c r="E14" t="s">
+        <v>77</v>
+      </c>
+      <c r="F14" t="s">
+        <v>78</v>
+      </c>
+      <c r="G14" t="s">
+        <v>49</v>
+      </c>
+      <c r="H14" t="s">
+        <v>55</v>
+      </c>
+      <c r="I14" t="s">
+        <v>13</v>
+      </c>
+      <c r="J14" t="s">
+        <v>74</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>